<commit_message>
Simplify row heading labels to "Row N" in KEYMAP docs
Drop the verbose, language-inconsistent parentheticals (QWERTY 上段 /
home row / Z row / thumb) and the leading "■" marker from the physical-row
heading cells, leaving just "Row 1".."Row 4". The highlighted heading-row
background is kept. Removes the now-redundant ROW_DESCRIPTIONS table since
the labels match the existing fallback.
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -652,7 +652,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -972,7 +972,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1162,7 +1162,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -1372,7 +1372,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -1502,7 +1502,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1692,7 +1692,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1842,7 +1842,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -2020,7 +2020,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -2262,7 +2262,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2528,7 +2528,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2686,7 +2686,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2856,7 +2856,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2982,7 +2982,7 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -3084,7 +3084,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -3182,7 +3182,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -3304,7 +3304,7 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -3394,7 +3394,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -3488,7 +3488,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -3578,7 +3578,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -3688,7 +3688,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3778,7 +3778,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3868,7 +3868,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3958,7 +3958,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -4068,7 +4068,7 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -4198,7 +4198,7 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -4288,7 +4288,7 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -4378,7 +4378,7 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -4488,7 +4488,7 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -4578,7 +4578,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -4668,7 +4668,7 @@
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -4758,7 +4758,7 @@
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4868,7 +4868,7 @@
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4974,7 +4974,7 @@
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -5196,7 +5196,7 @@
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -5310,7 +5310,7 @@
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -5536,7 +5536,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -5666,7 +5666,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -5856,7 +5856,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -6046,7 +6046,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -6256,7 +6256,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -6386,7 +6386,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -6576,7 +6576,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -6726,7 +6726,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -6904,7 +6904,7 @@
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -7154,7 +7154,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -7428,7 +7428,7 @@
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -7586,7 +7586,7 @@
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -7756,7 +7756,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -7890,7 +7890,7 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -7992,7 +7992,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -8090,7 +8090,7 @@
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -8212,7 +8212,7 @@
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -8302,7 +8302,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -8396,7 +8396,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -8486,7 +8486,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -8596,7 +8596,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -8686,7 +8686,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -8784,7 +8784,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -8882,7 +8882,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -8992,7 +8992,7 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -9122,7 +9122,7 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -9220,7 +9220,7 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
@@ -9318,7 +9318,7 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
@@ -9428,7 +9428,7 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -9542,7 +9542,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
@@ -9636,7 +9636,7 @@
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -9734,7 +9734,7 @@
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -9844,7 +9844,7 @@
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>■ Row 1 (QWERTY 上段)</t>
+          <t>Row 1</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -9950,7 +9950,7 @@
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>■ Row 2 (home row)</t>
+          <t>Row 2</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
@@ -10176,7 +10176,7 @@
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>■ Row 3 (Z row)</t>
+          <t>Row 3</t>
         </is>
       </c>
       <c r="B98" s="7" t="inlineStr">
@@ -10290,7 +10290,7 @@
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>■ Row 4 (thumb)</t>
+          <t>Row 4</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Rename operation label "単発タップ" to "タップ" in KEYMAP docs
Shorten the verbose single-tap operation label to just "タップ" in the
operation column of both the HTML and Excel tables. The string also serves
as the internal dispatch key in resolve(), so it is renamed uniformly;
the resolution logic and all other labels (ホールド / ダブルタップ /
Shift+ / Ctrl+) are unchanged.
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -722,7 +722,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -852,7 +852,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -1232,7 +1232,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1442,7 +1442,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -1572,7 +1572,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -1762,7 +1762,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1912,7 +1912,7 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr"/>
@@ -2090,7 +2090,7 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr"/>
@@ -2332,7 +2332,7 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -2598,7 +2598,7 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
@@ -2756,7 +2756,7 @@
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr"/>
@@ -2926,7 +2926,7 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr"/>
@@ -3052,7 +3052,7 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -3154,7 +3154,7 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -3252,7 +3252,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr"/>
@@ -3374,7 +3374,7 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr"/>
@@ -3464,7 +3464,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr"/>
@@ -3558,7 +3558,7 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr"/>
@@ -3648,7 +3648,7 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr"/>
@@ -3758,7 +3758,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr"/>
@@ -3848,7 +3848,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr"/>
@@ -3938,7 +3938,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr"/>
@@ -4028,7 +4028,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B72" s="9" t="inlineStr"/>
@@ -4138,7 +4138,7 @@
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
@@ -4268,7 +4268,7 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr"/>
@@ -4358,7 +4358,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B79" s="9" t="inlineStr"/>
@@ -4448,7 +4448,7 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B81" s="9" t="inlineStr"/>
@@ -4558,7 +4558,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr"/>
@@ -4648,7 +4648,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B86" s="9" t="inlineStr"/>
@@ -4738,7 +4738,7 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B88" s="9" t="inlineStr"/>
@@ -4828,7 +4828,7 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B90" s="9" t="inlineStr"/>
@@ -4938,7 +4938,7 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B93" s="9" t="inlineStr"/>
@@ -5044,7 +5044,7 @@
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B95" s="9" t="inlineStr">
@@ -5266,7 +5266,7 @@
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B99" s="9" t="inlineStr">
@@ -5380,7 +5380,7 @@
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B101" s="9" t="inlineStr"/>
@@ -5606,7 +5606,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -5736,7 +5736,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -5926,7 +5926,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -6116,7 +6116,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -6326,7 +6326,7 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
@@ -6456,7 +6456,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -6646,7 +6646,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -6796,7 +6796,7 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr"/>
@@ -6974,7 +6974,7 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr"/>
@@ -7224,7 +7224,7 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -7498,7 +7498,7 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
@@ -7656,7 +7656,7 @@
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr"/>
@@ -7826,7 +7826,7 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr"/>
@@ -7960,7 +7960,7 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B50" s="9" t="inlineStr">
@@ -8062,7 +8062,7 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
@@ -8160,7 +8160,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr"/>
@@ -8282,7 +8282,7 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr"/>
@@ -8372,7 +8372,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr"/>
@@ -8466,7 +8466,7 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr"/>
@@ -8556,7 +8556,7 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr"/>
@@ -8666,7 +8666,7 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr"/>
@@ -8756,7 +8756,7 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr"/>
@@ -8854,7 +8854,7 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr"/>
@@ -8952,7 +8952,7 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B72" s="9" t="inlineStr"/>
@@ -9062,7 +9062,7 @@
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
@@ -9192,7 +9192,7 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr"/>
@@ -9290,7 +9290,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B79" s="9" t="inlineStr"/>
@@ -9388,7 +9388,7 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B81" s="9" t="inlineStr"/>
@@ -9498,7 +9498,7 @@
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B84" s="9" t="inlineStr">
@@ -9612,7 +9612,7 @@
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B86" s="9" t="inlineStr">
@@ -9706,7 +9706,7 @@
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B88" s="9" t="inlineStr"/>
@@ -9804,7 +9804,7 @@
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B90" s="9" t="inlineStr"/>
@@ -9914,7 +9914,7 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B93" s="9" t="inlineStr"/>
@@ -10020,7 +10020,7 @@
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B95" s="9" t="inlineStr">
@@ -10246,7 +10246,7 @@
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B99" s="9" t="inlineStr">
@@ -10360,7 +10360,7 @@
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>単発タップ</t>
+          <t>タップ</t>
         </is>
       </c>
       <c r="B101" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: regenerate KEYMAP.html and KEYMAP.xlsx from keymap
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -545,12 +545,12 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
@@ -635,7 +635,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DEFAULT レイヤー</t>
+          <t>BASE_QWERTY レイヤー</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1215,32 +1215,32 @@
       <c r="E13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo SYMBOL</t>
+&amp;mo NUM_SYMBOL</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_1</t>
+&amp;mo VIM_NORMAL_BASE</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt SYMBOL ENTER</t>
+&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
@@ -1381,7 +1381,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>SYMBOL レイヤー</t>
+          <t>NUM_SYMBOL レイヤー</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
@@ -1905,13 +1905,13 @@
       <c r="E25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1924,7 +1924,7 @@
       <c r="I25" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_1 レイヤー</t>
+          <t>VIM_NORMAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
@@ -2674,7 +2674,7 @@
       <c r="D40" s="9" t="inlineStr"/>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>⇒VIM_VISUAL</t>
+          <t>⇒VIM_VISUAL_BASE</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -2720,7 +2720,7 @@
         <is>
           <t>HOME
 ▸ ⇧↓
-▸ ⇒VIM_VISUAL</t>
+▸ ⇒VIM_VISUAL_BASE</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -2784,7 +2784,7 @@
       <c r="G42" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2797,7 +2797,7 @@
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt VIM_NORMAL_2 ENTER</t>
+&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_2 レイヤー</t>
+          <t>VIM_NORMAL_SYM レイヤー</t>
         </is>
       </c>
       <c r="B45" s="4" t="n"/>
@@ -3356,7 +3356,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>MOUSE レイヤー</t>
+          <t>MOUSE_MOVE レイヤー</t>
         </is>
       </c>
       <c r="B55" s="4" t="n"/>
@@ -3517,7 +3517,7 @@
       <c r="L58" s="7" t="inlineStr">
         <is>
           <t>K
-&amp;mo SCROLL</t>
+&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
@@ -3750,7 +3750,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>SCROLL レイヤー</t>
+          <t>MOUSE_SCROLL レイヤー</t>
         </is>
       </c>
       <c r="B64" s="4" t="n"/>
@@ -4960,7 +4960,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>VIM_VISUAL レイヤー</t>
+          <t>VIM_VISUAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B91" s="4" t="n"/>
@@ -5075,7 +5075,7 @@
 ▸ RShift
 ▸ ⌃C
 ▸ →
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="K93" s="9" t="inlineStr"/>
@@ -5086,7 +5086,7 @@
           <t>LShift
 ▸ RShift
 ▸ ⌃V
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
           <t>LShift
 ▸ RShift
 ▸ ⌃X
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr"/>
@@ -5411,7 +5411,7 @@
           <t>LShift
 ▸ RShift
 ▸ ⌃X
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr"/>
@@ -5420,7 +5420,7 @@
           <t>LShift
 ▸ RShift
 ▸ →
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
@@ -5564,12 +5564,12 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
@@ -5654,7 +5654,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DEFAULT レイヤー</t>
+          <t>BASE_QWERTY レイヤー</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -6234,32 +6234,32 @@
       <c r="E13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo SYMBOL</t>
+&amp;mo NUM_SYMBOL</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_1</t>
+&amp;mo VIM_NORMAL_BASE</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt SYMBOL ENTER</t>
+&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
@@ -6300,28 +6300,28 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo SYMBOL</t>
+          <t>&amp;mo NUM_SYMBOL</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr"/>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo VIM_NORMAL_1</t>
+          <t>&amp;mo VIM_NORMAL_BASE</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt SYMBOL ENTER</t>
+          <t>&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr"/>
@@ -6360,12 +6360,12 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt SYMBOL ENTER</t>
+          <t>&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr"/>
@@ -6400,7 +6400,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>SYMBOL レイヤー</t>
+          <t>NUM_SYMBOL レイヤー</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
@@ -6924,13 +6924,13 @@
       <c r="E25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -6943,7 +6943,7 @@
       <c r="I25" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -6986,19 +6986,19 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr"/>
       <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo VIM_NORMAL_2</t>
+          <t>&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr"/>
@@ -7030,12 +7030,12 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr"/>
@@ -7058,7 +7058,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_1 レイヤー</t>
+          <t>VIM_NORMAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
@@ -7728,7 +7728,7 @@
       <c r="E40" s="10" t="inlineStr">
         <is>
           <t>mm_vim_v[0]
-▸ &amp;to VIM_VISUAL</t>
+▸ &amp;to VIM_VISUAL_BASE</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -7838,7 +7838,7 @@
       <c r="G42" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -7851,7 +7851,7 @@
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt VIM_NORMAL_2 ENTER</t>
+&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr"/>
@@ -7890,14 +7890,14 @@
       <c r="F43" s="9" t="inlineStr"/>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo VIM_NORMAL_2</t>
+          <t>&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="9" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 ENTER</t>
+          <t>&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K43" s="9" t="inlineStr"/>
@@ -7937,7 +7937,7 @@
       <c r="I44" s="9" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 ENTER</t>
+          <t>&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K44" s="9" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_2 レイヤー</t>
+          <t>VIM_NORMAL_SYM レイヤー</t>
         </is>
       </c>
       <c r="B45" s="4" t="n"/>
@@ -8422,7 +8422,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>MOUSE レイヤー</t>
+          <t>MOUSE_MOVE レイヤー</t>
         </is>
       </c>
       <c r="B55" s="4" t="n"/>
@@ -8583,7 +8583,7 @@
       <c r="L58" s="7" t="inlineStr">
         <is>
           <t>K
-&amp;mo SCROLL</t>
+&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
@@ -8617,7 +8617,7 @@
       <c r="K59" s="9" t="inlineStr"/>
       <c r="L59" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo SCROLL</t>
+          <t>&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="M59" s="9" t="inlineStr"/>
@@ -8816,7 +8816,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>SCROLL レイヤー</t>
+          <t>MOUSE_SCROLL レイヤー</t>
         </is>
       </c>
       <c r="B64" s="4" t="n"/>
@@ -10094,7 +10094,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>VIM_VISUAL レイヤー</t>
+          <t>VIM_VISUAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B91" s="4" t="n"/>

</xml_diff>

<commit_message>
refactor(keymap): clarify layer node and alias names (#13)
* refactor(keymap): clarify layer node and alias names

Rename layer node labels and #define aliases so each layer's role is
clear from its name:

- DEFAULT      -> BASE_QWERTY
- SYMBOL       -> NUM_SYMBOL
- VIM_NORMAL_1 -> VIM_NORMAL_BASE  (Vim normal for the BASE layer)
- VIM_NORMAL_2 -> VIM_NORMAL_SYM   (Vim normal for the SYM layer)
- MOUSE        -> MOUSE_MOVE
- SCROLL       -> MOUSE_SCROLL      (child layer of MOUSE_MOVE)
- VIM_VISUAL   -> VIM_VISUAL_BASE   (Vim visual for the BASE layer)

Aliases VIM_N1/VIM_N2/VISUAL renamed to VIM_BASE/VIM_SYM/VIM_VISUAL
and all &mo/&lt/&to references updated accordingly.

* docs: regenerate KEYMAP.html and KEYMAP.xlsx from keymap

---------

Co-authored-by: Claude <noreply@anthropic.com>
Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -545,12 +545,12 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
@@ -635,7 +635,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DEFAULT レイヤー</t>
+          <t>BASE_QWERTY レイヤー</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -1215,32 +1215,32 @@
       <c r="E13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo SYMBOL</t>
+&amp;mo NUM_SYMBOL</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_1</t>
+&amp;mo VIM_NORMAL_BASE</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt SYMBOL ENTER</t>
+&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
@@ -1381,7 +1381,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>SYMBOL レイヤー</t>
+          <t>NUM_SYMBOL レイヤー</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
@@ -1905,13 +1905,13 @@
       <c r="E25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1924,7 +1924,7 @@
       <c r="I25" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_1 レイヤー</t>
+          <t>VIM_NORMAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
@@ -2674,7 +2674,7 @@
       <c r="D40" s="9" t="inlineStr"/>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>⇒VIM_VISUAL</t>
+          <t>⇒VIM_VISUAL_BASE</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -2720,7 +2720,7 @@
         <is>
           <t>HOME
 ▸ ⇧↓
-▸ ⇒VIM_VISUAL</t>
+▸ ⇒VIM_VISUAL_BASE</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -2784,7 +2784,7 @@
       <c r="G42" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -2797,7 +2797,7 @@
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt VIM_NORMAL_2 ENTER</t>
+&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_2 レイヤー</t>
+          <t>VIM_NORMAL_SYM レイヤー</t>
         </is>
       </c>
       <c r="B45" s="4" t="n"/>
@@ -3356,7 +3356,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>MOUSE レイヤー</t>
+          <t>MOUSE_MOVE レイヤー</t>
         </is>
       </c>
       <c r="B55" s="4" t="n"/>
@@ -3517,7 +3517,7 @@
       <c r="L58" s="7" t="inlineStr">
         <is>
           <t>K
-&amp;mo SCROLL</t>
+&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
@@ -3750,7 +3750,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>SCROLL レイヤー</t>
+          <t>MOUSE_SCROLL レイヤー</t>
         </is>
       </c>
       <c r="B64" s="4" t="n"/>
@@ -4960,7 +4960,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>VIM_VISUAL レイヤー</t>
+          <t>VIM_VISUAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B91" s="4" t="n"/>
@@ -5075,7 +5075,7 @@
 ▸ RShift
 ▸ ⌃C
 ▸ →
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="K93" s="9" t="inlineStr"/>
@@ -5086,7 +5086,7 @@
           <t>LShift
 ▸ RShift
 ▸ ⌃V
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
           <t>LShift
 ▸ RShift
 ▸ ⌃X
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="E95" s="9" t="inlineStr"/>
@@ -5411,7 +5411,7 @@
           <t>LShift
 ▸ RShift
 ▸ ⌃X
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr"/>
@@ -5420,7 +5420,7 @@
           <t>LShift
 ▸ RShift
 ▸ →
-▸ ⇒DEFAULT</t>
+▸ ⇒BASE_QWERTY</t>
         </is>
       </c>
       <c r="F99" s="9" t="inlineStr">
@@ -5564,12 +5564,12 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
@@ -5654,7 +5654,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>DEFAULT レイヤー</t>
+          <t>BASE_QWERTY レイヤー</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -6234,32 +6234,32 @@
       <c r="E13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_1 SPACE</t>
+&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo SYMBOL</t>
+&amp;mo NUM_SYMBOL</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_1</t>
+&amp;mo VIM_NORMAL_BASE</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt SYMBOL ENTER</t>
+&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
@@ -6300,28 +6300,28 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo SYMBOL</t>
+          <t>&amp;mo NUM_SYMBOL</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr"/>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo VIM_NORMAL_1</t>
+          <t>&amp;mo VIM_NORMAL_BASE</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt SYMBOL ENTER</t>
+          <t>&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr"/>
@@ -6360,12 +6360,12 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_1 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_BASE SPACE</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt SYMBOL ENTER</t>
+          <t>&amp;lt NUM_SYMBOL ENTER</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr"/>
@@ -6400,7 +6400,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>SYMBOL レイヤー</t>
+          <t>NUM_SYMBOL レイヤー</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
@@ -6924,13 +6924,13 @@
       <c r="E25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>SPACE
-&amp;lt VIM_NORMAL_2 SPACE</t>
+&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -6943,7 +6943,7 @@
       <c r="I25" s="7" t="inlineStr">
         <is>
           <t>mo2
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -6986,19 +6986,19 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr"/>
       <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo VIM_NORMAL_2</t>
+          <t>&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr"/>
@@ -7030,12 +7030,12 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 SPACE</t>
+          <t>&amp;lt VIM_NORMAL_SYM SPACE</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr"/>
@@ -7058,7 +7058,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_1 レイヤー</t>
+          <t>VIM_NORMAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
@@ -7728,7 +7728,7 @@
       <c r="E40" s="10" t="inlineStr">
         <is>
           <t>mm_vim_v[0]
-▸ &amp;to VIM_VISUAL</t>
+▸ &amp;to VIM_VISUAL_BASE</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -7838,7 +7838,7 @@
       <c r="G42" s="7" t="inlineStr">
         <is>
           <t>mo1 (L center)
-&amp;mo VIM_NORMAL_2</t>
+&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr"/>
@@ -7851,7 +7851,7 @@
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>lt1 ENTER
-&amp;lt VIM_NORMAL_2 ENTER</t>
+&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr"/>
@@ -7890,14 +7890,14 @@
       <c r="F43" s="9" t="inlineStr"/>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo VIM_NORMAL_2</t>
+          <t>&amp;mo VIM_NORMAL_SYM</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="9" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 ENTER</t>
+          <t>&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K43" s="9" t="inlineStr"/>
@@ -7937,7 +7937,7 @@
       <c r="I44" s="9" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>&amp;lt VIM_NORMAL_2 ENTER</t>
+          <t>&amp;lt VIM_NORMAL_SYM ENTER</t>
         </is>
       </c>
       <c r="K44" s="9" t="inlineStr"/>
@@ -7952,7 +7952,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>VIM_NORMAL_2 レイヤー</t>
+          <t>VIM_NORMAL_SYM レイヤー</t>
         </is>
       </c>
       <c r="B45" s="4" t="n"/>
@@ -8422,7 +8422,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>MOUSE レイヤー</t>
+          <t>MOUSE_MOVE レイヤー</t>
         </is>
       </c>
       <c r="B55" s="4" t="n"/>
@@ -8583,7 +8583,7 @@
       <c r="L58" s="7" t="inlineStr">
         <is>
           <t>K
-&amp;mo SCROLL</t>
+&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
@@ -8617,7 +8617,7 @@
       <c r="K59" s="9" t="inlineStr"/>
       <c r="L59" s="9" t="inlineStr">
         <is>
-          <t>&amp;mo SCROLL</t>
+          <t>&amp;mo MOUSE_SCROLL</t>
         </is>
       </c>
       <c r="M59" s="9" t="inlineStr"/>
@@ -8816,7 +8816,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>SCROLL レイヤー</t>
+          <t>MOUSE_SCROLL レイヤー</t>
         </is>
       </c>
       <c r="B64" s="4" t="n"/>
@@ -10094,7 +10094,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>VIM_VISUAL レイヤー</t>
+          <t>VIM_VISUAL_BASE レイヤー</t>
         </is>
       </c>
       <c r="B91" s="4" t="n"/>

</xml_diff>